<commit_message>
fix: adjust brand spelling and supplier registration realism
Agent-Logs-Url: https://github.com/Setytlol/power_bi/sessions/7a47e2fd-aaba-4755-b971-b7e2b61c5028

Co-authored-by: Setytlol <81207521+Setytlol@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/dim_fornecedores.xlsx
+++ b/data/dim_fornecedores.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>441607790259</t>
+          <t>634895718</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>810117303572</t>
+          <t>523734972</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>919472468554</t>
+          <t>529389014</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -733,10 +733,10 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P4" s="1" t="n">
-        <v>46020</v>
+        <v>45236</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>651435606402</t>
+          <t>459525748</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -812,10 +812,10 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P5" s="1" t="n">
-        <v>45954</v>
+        <v>44786</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>554931713471</t>
+          <t>342285876</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -894,7 +894,7 @@
         <v>4</v>
       </c>
       <c r="P6" s="1" t="n">
-        <v>43122</v>
+        <v>45954</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>379307941680</t>
+          <t>103344769</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         <v>4</v>
       </c>
       <c r="P7" s="1" t="n">
-        <v>45848</v>
+        <v>43122</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>890157975566</t>
+          <t>130349564</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -1049,10 +1049,10 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P8" s="1" t="n">
-        <v>45000</v>
+        <v>43575</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>236251178483</t>
+          <t>580404538</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1128,10 +1128,10 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P9" s="1" t="n">
-        <v>43747</v>
+        <v>45848</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>87934225480</t>
+          <t>599770319</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1199,7 +1199,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1207,10 +1207,10 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="1" t="n">
-        <v>45536</v>
+        <v>45000</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>382204480059</t>
+          <t>161136438</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1286,10 +1286,10 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P11" s="1" t="n">
-        <v>45142</v>
+        <v>43747</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>34528312921</t>
+          <t>832395540</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1365,10 +1365,10 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P12" s="1" t="n">
-        <v>45240</v>
+        <v>45536</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>475480997051</t>
+          <t>925500248</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1436,7 +1436,7 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1444,10 +1444,10 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P13" s="1" t="n">
-        <v>45657</v>
+        <v>45142</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>30312468654</t>
+          <t>334564360</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P14" s="1" t="n">
-        <v>45056</v>
+        <v>45240</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>213398909031</t>
+          <t>916698734</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -1602,10 +1602,10 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P15" s="1" t="n">
-        <v>44122</v>
+        <v>45657</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>572223753013</t>
+          <t>457319431</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P16" s="1" t="n">
-        <v>44601</v>
+        <v>45354</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>819761371793</t>
+          <t>705850704</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>2</v>
       </c>
       <c r="P17" s="1" t="n">
-        <v>43302</v>
+        <v>44122</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>815828788451</t>
+          <t>186191493</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         <v>4</v>
       </c>
       <c r="P18" s="1" t="n">
-        <v>44117</v>
+        <v>44601</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>813246102055</t>
+          <t>496360081</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1910,7 +1910,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -1918,10 +1918,10 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P19" s="1" t="n">
-        <v>43438</v>
+        <v>43302</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>476105803060</t>
+          <t>722028733</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -1997,10 +1997,10 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P20" s="1" t="n">
-        <v>44281</v>
+        <v>44117</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>60939358252</t>
+          <t>423541287</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -2076,10 +2076,10 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P21" s="1" t="n">
-        <v>45669</v>
+        <v>43438</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>375458157952</t>
+          <t>270476398</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -2155,10 +2155,10 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P22" s="1" t="n">
-        <v>44623</v>
+        <v>44281</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>346752574087</t>
+          <t>324184334</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -2234,10 +2234,10 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P23" s="1" t="n">
-        <v>45437</v>
+        <v>45669</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>524404029444</t>
+          <t>195540567</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -2313,10 +2313,10 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P24" s="1" t="n">
-        <v>45189</v>
+        <v>45796</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>119771117958</t>
+          <t>123717335</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2384,7 +2384,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -2392,10 +2392,10 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P25" s="1" t="n">
-        <v>43603</v>
+        <v>45741</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>647217745725</t>
+          <t>272552610</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         <v>3</v>
       </c>
       <c r="P26" s="1" t="n">
-        <v>45832</v>
+        <v>44897</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2503,7 +2503,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>443661552597</t>
+          <t>857206505</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2542,7 +2542,7 @@
         </is>
       </c>
       <c r="M27" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -2550,10 +2550,10 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P27" s="1" t="n">
-        <v>45761</v>
+        <v>45189</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>750487672525</t>
+          <t>808496411</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="M28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -2632,7 +2632,7 @@
         <v>1</v>
       </c>
       <c r="P28" s="1" t="n">
-        <v>44129</v>
+        <v>44964</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>933121450742</t>
+          <t>956634123</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="M29" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -2708,10 +2708,10 @@
         </is>
       </c>
       <c r="O29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P29" s="1" t="n">
-        <v>43493</v>
+        <v>43603</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>886699537678</t>
+          <t>361917078</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2779,7 +2779,7 @@
         </is>
       </c>
       <c r="M30" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -2787,10 +2787,10 @@
         </is>
       </c>
       <c r="O30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P30" s="1" t="n">
-        <v>44585</v>
+        <v>45832</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>764739166014</t>
+          <t>690804839</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2858,7 +2858,7 @@
         </is>
       </c>
       <c r="M31" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2869,7 +2869,7 @@
         <v>1</v>
       </c>
       <c r="P31" s="1" t="n">
-        <v>43664</v>
+        <v>45761</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>566638684125</t>
+          <t>524831618</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="M32" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
         <v>5</v>
       </c>
       <c r="P32" s="1" t="n">
-        <v>44779</v>
+        <v>43603</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>731116581660</t>
+          <t>190053374</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3016,7 +3016,7 @@
         </is>
       </c>
       <c r="M33" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -3024,10 +3024,10 @@
         </is>
       </c>
       <c r="O33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P33" s="1" t="n">
-        <v>44284</v>
+        <v>43493</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>301992183738</t>
+          <t>862532878</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3095,18 +3095,18 @@
         </is>
       </c>
       <c r="M34" t="n">
+        <v>12</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
         <v>4</v>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>45 dias</t>
-        </is>
-      </c>
-      <c r="O34" t="n">
-        <v>2</v>
-      </c>
       <c r="P34" s="1" t="n">
-        <v>45705</v>
+        <v>44585</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>264813453496</t>
+          <t>966377394</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3174,7 +3174,7 @@
         </is>
       </c>
       <c r="M35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -3182,10 +3182,10 @@
         </is>
       </c>
       <c r="O35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P35" s="1" t="n">
-        <v>44152</v>
+        <v>43664</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>460462812971</t>
+          <t>371766524</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="M36" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -3261,10 +3261,10 @@
         </is>
       </c>
       <c r="O36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P36" s="1" t="n">
-        <v>45139</v>
+        <v>45379</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>392472311512</t>
+          <t>788839404</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -3340,10 +3340,10 @@
         </is>
       </c>
       <c r="O37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P37" s="1" t="n">
-        <v>44509</v>
+        <v>43641</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>518277883418</t>
+          <t>928299788</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="M38" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -3419,10 +3419,10 @@
         </is>
       </c>
       <c r="O38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P38" s="1" t="n">
-        <v>44383</v>
+        <v>44920</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>438893855685</t>
+          <t>871795521</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3490,7 +3490,7 @@
         </is>
       </c>
       <c r="M39" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -3498,10 +3498,10 @@
         </is>
       </c>
       <c r="O39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P39" s="1" t="n">
-        <v>43749</v>
+        <v>44698</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -3530,7 +3530,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>263046950820</t>
+          <t>672964792</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3569,7 +3569,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -3577,10 +3577,10 @@
         </is>
       </c>
       <c r="O40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P40" s="1" t="n">
-        <v>44358</v>
+        <v>44152</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>735587918743</t>
+          <t>901312299</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3648,7 +3648,7 @@
         </is>
       </c>
       <c r="M41" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -3656,10 +3656,10 @@
         </is>
       </c>
       <c r="O41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P41" s="1" t="n">
-        <v>44732</v>
+        <v>45139</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>

</xml_diff>